<commit_message>
Map reject-class rules and review decisions
</commit_message>
<xml_diff>
--- a/config/rules_structured.xlsx
+++ b/config/rules_structured.xlsx
@@ -460,7 +460,11 @@
       <c r="C2" t="b">
         <v>1</v>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>拒收类/不建议接收类；无许可资质、无处置能力或规则列明不可接收的爆炸物、医疗废物、放射性元素，以及含铅、汞、铊、铍等试剂。</t>
+        </is>
+      </c>
       <c r="E2" t="b">
         <v>1</v>
       </c>
@@ -477,7 +481,11 @@
       <c r="C3" t="b">
         <v>1</v>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>剧毒品专项规则；需人工复核，不作为 ERP 物化特性自动写入。</t>
+        </is>
+      </c>
       <c r="E3" t="b">
         <v>1</v>
       </c>
@@ -732,7 +740,11 @@
       <c r="C18" t="b">
         <v>1</v>
       </c>
-      <c r="D18" t="inlineStr"/>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>未知、无标签、无 MSDS 或无法辨识；需人工复核。</t>
+        </is>
+      </c>
       <c r="E18" t="b">
         <v>1</v>
       </c>
@@ -4188,7 +4200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F390"/>
+  <dimension ref="A1:F419"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14336,6 +14348,876 @@
         </is>
       </c>
       <c r="F390" t="inlineStr"/>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>拒收类</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D391" t="b">
+        <v>1</v>
+      </c>
+      <c r="E391" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F391" t="inlineStr">
+        <is>
+          <t>业务别名：拒收类等同于不建议接收类</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>黑索今</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D392" t="b">
+        <v>1</v>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F392" t="inlineStr">
+        <is>
+          <t>RDX / 环三亚甲基三硝胺</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>RDX</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D393" t="b">
+        <v>1</v>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F393" t="inlineStr">
+        <is>
+          <t>工业黑索今</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>环三亚甲基三硝胺</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D394" t="b">
+        <v>1</v>
+      </c>
+      <c r="E394" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F394" t="inlineStr">
+        <is>
+          <t>工业黑索今 RDX</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>太安</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D395" t="b">
+        <v>1</v>
+      </c>
+      <c r="E395" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F395" t="inlineStr">
+        <is>
+          <t>PETN / 季戊四醇四硝酸酯</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>PETN</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D396" t="b">
+        <v>1</v>
+      </c>
+      <c r="E396" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F396" t="inlineStr">
+        <is>
+          <t>太安</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>季戊四醇四硝酸酯</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D397" t="b">
+        <v>1</v>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F397" t="inlineStr">
+        <is>
+          <t>太安 PETN</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>奥克托今</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D398" t="b">
+        <v>1</v>
+      </c>
+      <c r="E398" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F398" t="inlineStr">
+        <is>
+          <t>HMX</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>HMX</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D399" t="b">
+        <v>1</v>
+      </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F399" t="inlineStr">
+        <is>
+          <t>奥克托今</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>特屈拉辛</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D400" t="b">
+        <v>1</v>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F400" t="inlineStr">
+        <is>
+          <t>炸药</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>炸药</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D401" t="b">
+        <v>1</v>
+      </c>
+      <c r="E401" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F401" t="inlineStr">
+        <is>
+          <t>无许可资质、无处置能力</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>医疗废物</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D402" t="b">
+        <v>1</v>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F402" t="inlineStr">
+        <is>
+          <t>血清、动物体内导出等医疗废物</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>放射性元素</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D403" t="b">
+        <v>1</v>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F403" t="inlineStr">
+        <is>
+          <t>氚、镭、铀等放射性元素</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>氚</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="D404" t="b">
+        <v>1</v>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F404" t="inlineStr">
+        <is>
+          <t>放射性元素</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>镭</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="D405" t="b">
+        <v>1</v>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F405" t="inlineStr">
+        <is>
+          <t>放射性元素</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>铀</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="D406" t="b">
+        <v>1</v>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F406" t="inlineStr">
+        <is>
+          <t>放射性元素</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>硝酸汞</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="D407" t="b">
+        <v>1</v>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F407" t="inlineStr">
+        <is>
+          <t>含铅、汞、铊、铍等拒收类举例</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>碘化汞</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="D408" t="b">
+        <v>1</v>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F408" t="inlineStr">
+        <is>
+          <t>含铅、汞、铊、铍等拒收类举例</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>溴化汞</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="D409" t="b">
+        <v>1</v>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F409" t="inlineStr">
+        <is>
+          <t>含铅、汞、铊、铍等拒收类举例</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>氰化汞</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="D410" t="b">
+        <v>1</v>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F410" t="inlineStr">
+        <is>
+          <t>含铅、汞、铊、铍等拒收类举例</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>硫氰酸汞</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="D411" t="b">
+        <v>1</v>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F411" t="inlineStr">
+        <is>
+          <t>含铅、汞、铊、铍等拒收类举例</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>氯化甲氧基乙基汞</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="D412" t="b">
+        <v>1</v>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F412" t="inlineStr">
+        <is>
+          <t>含铅、汞、铊、铍等拒收类举例</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>铊</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="D413" t="b">
+        <v>1</v>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F413" t="inlineStr">
+        <is>
+          <t>含铅、汞、铊、铍等拒收类举例</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>氧化亚铊</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="D414" t="b">
+        <v>1</v>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F414" t="inlineStr">
+        <is>
+          <t>含铅、汞、铊、铍等拒收类举例</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>氧化铊</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="D415" t="b">
+        <v>1</v>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F415" t="inlineStr">
+        <is>
+          <t>含铅、汞、铊、铍等拒收类举例</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>碳酸亚铊</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="D416" t="b">
+        <v>1</v>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F416" t="inlineStr">
+        <is>
+          <t>含铅、汞、铊、铍等拒收类举例</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>乙酸亚铊</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="D417" t="b">
+        <v>1</v>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F417" t="inlineStr">
+        <is>
+          <t>含铅、汞、铊、铍等拒收类举例</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>丙二酸铊</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="D418" t="b">
+        <v>1</v>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F418" t="inlineStr">
+        <is>
+          <t>含铅、汞、铊、铍等拒收类举例</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>不建议接收类</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>铍类</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D419" t="b">
+        <v>1</v>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F419" t="inlineStr">
+        <is>
+          <t>含铅、汞、铊、铍等拒收类举例</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14566,7 +15448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14613,6 +15495,26 @@
         <v>1</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NOTE-REJECT-001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>拒收类是业务处置结论，在 ERP 物化特性下拉中无对应可写选项；程序按“不建议接收类”识别并进入人工复核/不可自动写入。</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Classify dichromates and permanganates as oxidizers
</commit_message>
<xml_diff>
--- a/config/rules_structured.xlsx
+++ b/config/rules_structured.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="categories" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="rules" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="examples" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="aliases" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="thresholds" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="notes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="categories" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="rules" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="examples" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="aliases" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="thresholds" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="notes" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4200,7 +4200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F419"/>
+  <dimension ref="A1:F424"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7134,7 +7134,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>exact</t>
+          <t>contains</t>
         </is>
       </c>
       <c r="D113" t="b">
@@ -7145,7 +7145,11 @@
           <t>rules.xlsx</t>
         </is>
       </c>
-      <c r="F113" t="inlineStr"/>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>标准化氧化剂示例：重铬酸盐</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -15216,6 +15220,156 @@
       <c r="F419" t="inlineStr">
         <is>
           <t>含铅、汞、铊、铍等拒收类举例</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>氧化剂</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>高锰酸钾</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D420" t="b">
+        <v>1</v>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F420" t="inlineStr">
+        <is>
+          <t>标准化氧化剂示例：高锰酸盐</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>氧化剂</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>高锰酸钠</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D421" t="b">
+        <v>1</v>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F421" t="inlineStr">
+        <is>
+          <t>标准化氧化剂示例：高锰酸盐</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>氧化剂</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>高锰酸盐</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D422" t="b">
+        <v>1</v>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F422" t="inlineStr">
+        <is>
+          <t>标准化氧化剂示例：高锰酸盐</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>氧化剂</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>重铬酸钾</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D423" t="b">
+        <v>1</v>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F423" t="inlineStr">
+        <is>
+          <t>标准化氧化剂示例：重铬酸盐</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>氧化剂</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>重铬酸盐</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>contains</t>
+        </is>
+      </c>
+      <c r="D424" t="b">
+        <v>1</v>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>rules.xlsx</t>
+        </is>
+      </c>
+      <c r="F424" t="inlineStr">
+        <is>
+          <t>标准化氧化剂示例：重铬酸盐</t>
         </is>
       </c>
     </row>

</xml_diff>